<commit_message>
added tests for r17
</commit_message>
<xml_diff>
--- a/docs/4. HACKATHON_FRAML_RULES.xlsx
+++ b/docs/4. HACKATHON_FRAML_RULES.xlsx
@@ -1245,7 +1245,7 @@
       <charset val="238"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1286,6 +1286,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFBF00"/>
         <bgColor rgb="FFFF9900"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FF993300"/>
       </patternFill>
     </fill>
   </fills>
@@ -1358,7 +1364,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1503,16 +1509,24 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -2176,37 +2190,37 @@
         <v>75</v>
       </c>
     </row>
-    <row r="11" s="16" customFormat="true" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
+    <row r="11" s="29" customFormat="true" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="25" t="s">
         <v>78</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12" t="n">
+      <c r="F11" s="36"/>
+      <c r="G11" s="27" t="n">
         <v>15</v>
       </c>
-      <c r="H11" s="12" t="s">
+      <c r="H11" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="I11" s="10" t="s">
+      <c r="I11" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="J11" s="10" t="s">
+      <c r="J11" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="K11" s="10"/>
-      <c r="L11" s="15" t="s">
+      <c r="K11" s="25"/>
+      <c r="L11" s="37" t="s">
         <v>82</v>
       </c>
     </row>
@@ -2265,7 +2279,7 @@
       <c r="F13" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="G13" s="36" t="n">
+      <c r="G13" s="38" t="n">
         <v>20</v>
       </c>
       <c r="H13" s="22" t="s">
@@ -2274,7 +2288,7 @@
       <c r="I13" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="J13" s="37" t="s">
+      <c r="J13" s="39" t="s">
         <v>93</v>
       </c>
       <c r="K13" s="19" t="s">
@@ -2343,17 +2357,17 @@
       <c r="H15" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="I15" s="31" t="s">
+      <c r="I15" s="40" t="s">
         <v>105</v>
       </c>
       <c r="J15" s="25"/>
       <c r="K15" s="25"/>
-      <c r="L15" s="38" t="s">
+      <c r="L15" s="37" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C17" s="39" t="s">
+      <c r="C17" s="41" t="s">
         <v>107</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added tests to r18
</commit_message>
<xml_diff>
--- a/docs/4. HACKATHON_FRAML_RULES.xlsx
+++ b/docs/4. HACKATHON_FRAML_RULES.xlsx
@@ -2224,39 +2224,39 @@
         <v>82</v>
       </c>
     </row>
-    <row r="12" s="16" customFormat="true" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="s">
+    <row r="12" s="29" customFormat="true" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="D12" s="26" t="s">
         <v>85</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="F12" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="G12" s="12" t="n">
+      <c r="G12" s="27" t="n">
         <v>3</v>
       </c>
-      <c r="H12" s="12" t="s">
+      <c r="H12" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="I12" s="10" t="s">
+      <c r="I12" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="J12" s="10" t="s">
+      <c r="J12" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="K12" s="10"/>
-      <c r="L12" s="13" t="s">
+      <c r="K12" s="25"/>
+      <c r="L12" s="28" t="s">
         <v>88</v>
       </c>
     </row>

</xml_diff>